<commit_message>
add multilingual and voice input/output support
</commit_message>
<xml_diff>
--- a/data/official_data/knowledge/university_info.xlsx
+++ b/data/official_data/knowledge/university_info.xlsx
@@ -1026,13 +1026,13 @@
       <c r="A23" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="6" t="s">
         <v>59</v>
       </c>
       <c r="E23" s="5" t="s">

</xml_diff>